<commit_message>
Fix: ensure no digits are removed from phone numbers
</commit_message>
<xml_diff>
--- a/ophtalmologues_zone3.xlsx
+++ b/ophtalmologues_zone3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15538" uniqueCount="2584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16196" uniqueCount="2766">
   <si>
     <t>PROSPECTS</t>
   </si>
@@ -7764,6 +7764,552 @@
   </si>
   <si>
     <t>https://www.pagesjaunes.fr/pros/62295866</t>
+  </si>
+  <si>
+    <t>Tulle</t>
+  </si>
+  <si>
+    <t>Laura Ghiorghiu</t>
+  </si>
+  <si>
+    <t>0555295775</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/tulle/laura-ghiorghiu-tulle</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/55570864</t>
+  </si>
+  <si>
+    <t>Dominique Gautier</t>
+  </si>
+  <si>
+    <t>0555230629</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/dominique-gautier-09043a14b</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde/dominique-gautier</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/04534768</t>
+  </si>
+  <si>
+    <t>Gautier Dominique Et Liozon Patrick SCM</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/dominique-gautier-4072a49</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/04674755</t>
+  </si>
+  <si>
+    <t>Hélène Barbara</t>
+  </si>
+  <si>
+    <t>0555170250</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde/helene-barbara</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/09443001</t>
+  </si>
+  <si>
+    <t>CENTRE HOSPITALIER DUBOIS BRIVE</t>
+  </si>
+  <si>
+    <t>0555926000</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/antoine-garcia-0299b57b</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/60522112</t>
+  </si>
+  <si>
+    <t>0555926004</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62633111</t>
+  </si>
+  <si>
+    <t>BRAKBI Fathia</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/53337141</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/63395925</t>
+  </si>
+  <si>
+    <t>Ussel</t>
+  </si>
+  <si>
+    <t>VINCENT JEAN PATRICE</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/jean-patrice-vincent-1978a9108</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/ussel/jean-patrice-vincent-ussel</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/60674836</t>
+  </si>
+  <si>
+    <t>Malemort</t>
+  </si>
+  <si>
+    <t>Sofiane Laribi</t>
+  </si>
+  <si>
+    <t>0555742538</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/sofianelaribi</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde/sofiane-laribi-brive-la-gaillarde</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/58832600</t>
+  </si>
+  <si>
+    <t>Demerliac Mailys</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62314508</t>
+  </si>
+  <si>
+    <t>REMI SERVANTIE</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde/remi-servantie-73ea848b-36de-4aa4-be14-61094452b7bb</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62585393</t>
+  </si>
+  <si>
+    <t>Laëtitia Boivin</t>
+  </si>
+  <si>
+    <t>0802012015</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/la%C3%ABtitia-boivin-438238233</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57536418</t>
+  </si>
+  <si>
+    <t>Rémi Servantie</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57786633</t>
+  </si>
+  <si>
+    <t>Kechaou Mohamed</t>
+  </si>
+  <si>
+    <t>0544403676</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/saint-mexant/habib-kechaou</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62092200</t>
+  </si>
+  <si>
+    <t>François Xavier Brousseaud</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/fran%C3%A7ois-xavier-bourmaud-2989a5b</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/malemort-sur-correze/francois-xavier-brousseaud</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57784002</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/laetitia-boivin-3a3939336</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57786631</t>
+  </si>
+  <si>
+    <t>HUGE LAURENT</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/ussel/laurent-huge-ussel</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/60674851</t>
+  </si>
+  <si>
+    <t>LARIBI SOFIANE</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/sofiane-laribi-06869a198</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/59880513</t>
+  </si>
+  <si>
+    <t>Thea Breuil</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/malemort/thea-breuil</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/64640630</t>
+  </si>
+  <si>
+    <t>Claudine Billot</t>
+  </si>
+  <si>
+    <t>0555231858</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/claudine-billot-77074372</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/63865372</t>
+  </si>
+  <si>
+    <t>HELENE BARBARA</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62575070</t>
+  </si>
+  <si>
+    <t>Brousseaud Francois Xavier</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/fran%C3%A7ois-xavier-brosseau-218931244</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/brive-la-gaillarde/francois-xavier-brousseaud-brive-la-gaillarde-19100</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62250806</t>
+  </si>
+  <si>
+    <t>Chamberet</t>
+  </si>
+  <si>
+    <t>Gautier Dominique</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/dominique-gautier-69a90848</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/chamberet/dominique-gautier-3524a9d0-8623-4839-85c5-7ee18e8bf5c3</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/60190289</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/sofiane-laribi-4446072ba</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/63648125</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/64638228</t>
+  </si>
+  <si>
+    <t>Arnac Pompadour</t>
+  </si>
+  <si>
+    <t>MADAME DEMERLIAC MAILYS</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/arnac-pompadour/mailys-demerliac-arnac-pompadour-19230</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/64340555</t>
+  </si>
+  <si>
+    <t>Remi Servantie</t>
+  </si>
+  <si>
+    <t>0555297900</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/tulle/remi-servantie</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/64626534</t>
+  </si>
+  <si>
+    <t>Creuse</t>
+  </si>
+  <si>
+    <t>La Souterraine</t>
+  </si>
+  <si>
+    <t>Jean-Paul Mousnier</t>
+  </si>
+  <si>
+    <t>0555632785</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/jeanne-mousnier-258380345</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/la-souterraine/jean-paul-mousnier</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/04610452</t>
+  </si>
+  <si>
+    <t>Guéret</t>
+  </si>
+  <si>
+    <t>Loïc Bourmault</t>
+  </si>
+  <si>
+    <t>0555518937</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/gueret/loic-bourmault-gueret-23011</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57808394</t>
+  </si>
+  <si>
+    <t>Aubusson</t>
+  </si>
+  <si>
+    <t>Yohan Benayoun</t>
+  </si>
+  <si>
+    <t>0555835050</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/yohan-benayoun</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/limoges/yohan-benayoun-limoges-cedex</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57660791</t>
+  </si>
+  <si>
+    <t>0001512015</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/fabien-petellat-72647932</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/gueret/fabien-petellat-gueret</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57614688</t>
+  </si>
+  <si>
+    <t>Lathiere Thomas</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/thomas-lathiere-7900a0223</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/gueret/thomas-lathiere-gueret</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/59879350</t>
+  </si>
+  <si>
+    <t>Vergne Benoit</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/benoit-vergne-534640128</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/paris/benoit-vergne</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57792880</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/gueret/yohan-benayoun-gueret-23000</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57661846</t>
+  </si>
+  <si>
+    <t>Quilbe Sebastien</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/chateauroux/sebastien-quilbe</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/60874365</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/francis-van-coppenolle-44941a6a</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/limoges/francis-van-coppenolle-limoges-cedex-1-87039</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57435550</t>
+  </si>
+  <si>
+    <t>Crocq</t>
+  </si>
+  <si>
+    <t>BENOIT VERGNE</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/62592456</t>
+  </si>
+  <si>
+    <t>Dordogne</t>
+  </si>
+  <si>
+    <t>Bergerac</t>
+  </si>
+  <si>
+    <t>Ilyana Ilieva</t>
+  </si>
+  <si>
+    <t>0553580956</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/ilyana-ilieva-1379273b7</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/bergerac/ilyana-ilieva</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/51879207</t>
+  </si>
+  <si>
+    <t>Le Bugue</t>
+  </si>
+  <si>
+    <t>Maxime Fat Cheung</t>
+  </si>
+  <si>
+    <t>0553048734</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/maxime-cheung-706717201</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/06742713</t>
+  </si>
+  <si>
+    <t>Boulazac Isle Manoire</t>
+  </si>
+  <si>
+    <t>Brian Redmill</t>
+  </si>
+  <si>
+    <t>0553355022</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/perigueux/brian-redmill-perigueux</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57777907</t>
+  </si>
+  <si>
+    <t>Trélissac</t>
+  </si>
+  <si>
+    <t>Isabelle Baylac-Fresno</t>
+  </si>
+  <si>
+    <t>0553454110</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/excideuil/isabelle-baylac-fresno</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/04539316</t>
+  </si>
+  <si>
+    <t>Champcevinel</t>
+  </si>
+  <si>
+    <t>Perin Laurent</t>
+  </si>
+  <si>
+    <t>0553049250</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/laurent-p%C3%A9rin-010459111</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/champcevinel/laurent-perin</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/59872575</t>
+  </si>
+  <si>
+    <t>Creysse</t>
+  </si>
+  <si>
+    <t>Jean Claude Geneau</t>
+  </si>
+  <si>
+    <t>0553235670</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/jeanne-geneau-b46677262</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/libourne/jean-claude-geneau</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57884036</t>
+  </si>
+  <si>
+    <t>Périgueux</t>
+  </si>
+  <si>
+    <t>Lam Delphine</t>
+  </si>
+  <si>
+    <t>0553021616</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/perigueux/delphine-lam-perigueux</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/61398576</t>
+  </si>
+  <si>
+    <t>Jean-Jacques Francerie</t>
+  </si>
+  <si>
+    <t>0533092645</t>
+  </si>
+  <si>
+    <t>https://fr.linkedin.com/in/jean-jacques-sulman-a9345224</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/champcevinel/jean-jacques-francerie-trelissac</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57622092</t>
+  </si>
+  <si>
+    <t>Magda Brosteanu</t>
+  </si>
+  <si>
+    <t>https://www.doctolib.fr/ophtalmologue/bergerac/magda-brosteanu</t>
+  </si>
+  <si>
+    <t>https://www.pagesjaunes.fr/pros/57459948</t>
   </si>
 </sst>
 </file>
@@ -8144,7 +8690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:V1111"/>
+  <dimension ref="B2:V1158"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="2" spans="2:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -56981,6 +57527,2074 @@
         <v>2583</v>
       </c>
     </row>
+    <row r="1112" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1112" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1112" t="s">
+        <v>2584</v>
+      </c>
+      <c r="D1112" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1112" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1112" t="s">
+        <v>2586</v>
+      </c>
+      <c r="P1112" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1112" t="s">
+        <v>2587</v>
+      </c>
+      <c r="U1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1112" t="s">
+        <v>2588</v>
+      </c>
+    </row>
+    <row r="1113" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1113" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1113" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1113" t="s">
+        <v>2589</v>
+      </c>
+      <c r="E1113" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1113" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1113" t="s">
+        <v>2589</v>
+      </c>
+      <c r="H1113" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1113" t="s">
+        <v>2590</v>
+      </c>
+      <c r="P1113" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1113" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1113" t="s">
+        <v>2591</v>
+      </c>
+      <c r="T1113" t="s">
+        <v>2592</v>
+      </c>
+      <c r="U1113" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1113" t="s">
+        <v>2593</v>
+      </c>
+    </row>
+    <row r="1114" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1114" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1114" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1114" t="s">
+        <v>2594</v>
+      </c>
+      <c r="E1114" t="s">
+        <v>2580</v>
+      </c>
+      <c r="F1114" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1114" t="s">
+        <v>2594</v>
+      </c>
+      <c r="H1114" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1114" t="s">
+        <v>2590</v>
+      </c>
+      <c r="P1114" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1114" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1114" t="s">
+        <v>2595</v>
+      </c>
+      <c r="T1114" t="s">
+        <v>2592</v>
+      </c>
+      <c r="U1114" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1114" t="s">
+        <v>2596</v>
+      </c>
+    </row>
+    <row r="1115" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1115" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1115" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1115" t="s">
+        <v>2597</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1115" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1115" t="s">
+        <v>2598</v>
+      </c>
+      <c r="P1115" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1115" t="s">
+        <v>2599</v>
+      </c>
+      <c r="U1115" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1115" t="s">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="1116" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1116" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1116" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1116" t="s">
+        <v>2601</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1116" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1116" t="s">
+        <v>2601</v>
+      </c>
+      <c r="H1116" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1116" t="s">
+        <v>2602</v>
+      </c>
+      <c r="P1116" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1116" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1116" t="s">
+        <v>2603</v>
+      </c>
+      <c r="T1116" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1116" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1116" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="1117" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1117" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1117" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1117" t="s">
+        <v>2580</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1117" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1117" t="s">
+        <v>2605</v>
+      </c>
+      <c r="P1117" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1117" t="s">
+        <v>2606</v>
+      </c>
+      <c r="U1117" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1117" t="s">
+        <v>2607</v>
+      </c>
+    </row>
+    <row r="1118" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1118" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1118" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1118" t="s">
+        <v>2608</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1118" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1118" t="s">
+        <v>2605</v>
+      </c>
+      <c r="P1118" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1118" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1118" t="s">
+        <v>2609</v>
+      </c>
+    </row>
+    <row r="1119" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1119" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1119" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1119" t="s">
+        <v>2579</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1119" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1119" t="s">
+        <v>2581</v>
+      </c>
+      <c r="P1119" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1119" t="s">
+        <v>2582</v>
+      </c>
+      <c r="U1119" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1119" t="s">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="1120" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1120" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1120" t="s">
+        <v>2611</v>
+      </c>
+      <c r="D1120" t="s">
+        <v>2612</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1120" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1120" t="s">
+        <v>2612</v>
+      </c>
+      <c r="H1120" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1120" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1120" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1120" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1120" t="s">
+        <v>2613</v>
+      </c>
+      <c r="T1120" t="s">
+        <v>2614</v>
+      </c>
+      <c r="U1120" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1120" t="s">
+        <v>2615</v>
+      </c>
+    </row>
+    <row r="1121" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1121" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1121" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1121" t="s">
+        <v>2617</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1121" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1121" t="s">
+        <v>2617</v>
+      </c>
+      <c r="H1121" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1121" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1121" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1121" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1121" t="s">
+        <v>2619</v>
+      </c>
+      <c r="T1121" t="s">
+        <v>2620</v>
+      </c>
+      <c r="U1121" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1121" t="s">
+        <v>2621</v>
+      </c>
+    </row>
+    <row r="1122" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1122" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1122" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1122" t="s">
+        <v>2622</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1122" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1122" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1122" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1122" t="s">
+        <v>2582</v>
+      </c>
+      <c r="U1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1122" t="s">
+        <v>2623</v>
+      </c>
+    </row>
+    <row r="1123" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1123" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1123" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1123" t="s">
+        <v>2624</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1123" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1123" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1123" t="s">
+        <v>2625</v>
+      </c>
+      <c r="U1123" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1123" t="s">
+        <v>2626</v>
+      </c>
+    </row>
+    <row r="1124" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1124" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1124" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1124" t="s">
+        <v>2627</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1124" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1124" t="s">
+        <v>2627</v>
+      </c>
+      <c r="H1124" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1124" t="s">
+        <v>2628</v>
+      </c>
+      <c r="P1124" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1124" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1124" t="s">
+        <v>2629</v>
+      </c>
+      <c r="T1124" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1124" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1124" t="s">
+        <v>2630</v>
+      </c>
+    </row>
+    <row r="1125" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1125" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1125" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1125" t="s">
+        <v>2631</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1125" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1125" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1125" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1125" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1125" t="s">
+        <v>2632</v>
+      </c>
+    </row>
+    <row r="1126" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1126" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1126" t="s">
+        <v>2567</v>
+      </c>
+      <c r="D1126" t="s">
+        <v>2633</v>
+      </c>
+      <c r="E1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1126" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1126" t="s">
+        <v>2634</v>
+      </c>
+      <c r="P1126" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1126" t="s">
+        <v>2635</v>
+      </c>
+      <c r="U1126" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1126" t="s">
+        <v>2636</v>
+      </c>
+    </row>
+    <row r="1127" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1127" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1127" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1127" t="s">
+        <v>2637</v>
+      </c>
+      <c r="E1127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1127" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1127" t="s">
+        <v>2637</v>
+      </c>
+      <c r="H1127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1127" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1127" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1127" t="s">
+        <v>2638</v>
+      </c>
+      <c r="T1127" t="s">
+        <v>2639</v>
+      </c>
+      <c r="U1127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1127" t="s">
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="1128" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1128" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1128" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1128" t="s">
+        <v>2627</v>
+      </c>
+      <c r="E1128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1128" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1128" t="s">
+        <v>2627</v>
+      </c>
+      <c r="H1128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1128" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1128" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1128" t="s">
+        <v>2641</v>
+      </c>
+      <c r="T1128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1128" t="s">
+        <v>2642</v>
+      </c>
+    </row>
+    <row r="1129" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1129" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1129" t="s">
+        <v>2611</v>
+      </c>
+      <c r="D1129" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1129" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1129" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1129" t="s">
+        <v>2644</v>
+      </c>
+      <c r="U1129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1129" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="1130" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1130" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1130" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1130" t="s">
+        <v>2646</v>
+      </c>
+      <c r="E1130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1130" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1130" t="s">
+        <v>2646</v>
+      </c>
+      <c r="H1130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1130" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1130" t="s">
+        <v>2647</v>
+      </c>
+      <c r="T1130" t="s">
+        <v>2620</v>
+      </c>
+      <c r="U1130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1130" t="s">
+        <v>2648</v>
+      </c>
+    </row>
+    <row r="1131" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1131" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1131" t="s">
+        <v>2616</v>
+      </c>
+      <c r="D1131" t="s">
+        <v>2649</v>
+      </c>
+      <c r="E1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1131" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1131" t="s">
+        <v>2618</v>
+      </c>
+      <c r="P1131" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1131" t="s">
+        <v>2650</v>
+      </c>
+      <c r="U1131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1131" t="s">
+        <v>2651</v>
+      </c>
+    </row>
+    <row r="1132" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1132" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1132" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1132" t="s">
+        <v>2652</v>
+      </c>
+      <c r="E1132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1132" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1132" t="s">
+        <v>2652</v>
+      </c>
+      <c r="H1132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1132" t="s">
+        <v>2653</v>
+      </c>
+      <c r="P1132" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1132" t="s">
+        <v>2654</v>
+      </c>
+      <c r="T1132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1132" t="s">
+        <v>2655</v>
+      </c>
+    </row>
+    <row r="1133" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1133" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1133" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1133" t="s">
+        <v>2656</v>
+      </c>
+      <c r="E1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1133" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1133" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1133" t="s">
+        <v>2599</v>
+      </c>
+      <c r="U1133" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1133" t="s">
+        <v>2657</v>
+      </c>
+    </row>
+    <row r="1134" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1134" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1134" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1134" t="s">
+        <v>2658</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1134" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1134" t="s">
+        <v>2658</v>
+      </c>
+      <c r="H1134" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1134" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1134" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1134" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1134" t="s">
+        <v>2659</v>
+      </c>
+      <c r="T1134" t="s">
+        <v>2660</v>
+      </c>
+      <c r="U1134" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1134" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="1135" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1135" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1135" t="s">
+        <v>2662</v>
+      </c>
+      <c r="D1135" t="s">
+        <v>2663</v>
+      </c>
+      <c r="E1135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1135" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1135" t="s">
+        <v>2663</v>
+      </c>
+      <c r="H1135" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1135" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1135" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1135" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1135" t="s">
+        <v>2664</v>
+      </c>
+      <c r="T1135" t="s">
+        <v>2665</v>
+      </c>
+      <c r="U1135" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1135" t="s">
+        <v>2666</v>
+      </c>
+    </row>
+    <row r="1136" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1136" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1136" t="s">
+        <v>2573</v>
+      </c>
+      <c r="D1136" t="s">
+        <v>2617</v>
+      </c>
+      <c r="E1136" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1136" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1136" t="s">
+        <v>2617</v>
+      </c>
+      <c r="H1136" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1136" t="s">
+        <v>2581</v>
+      </c>
+      <c r="P1136" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1136" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1136" t="s">
+        <v>2667</v>
+      </c>
+      <c r="T1136" t="s">
+        <v>2620</v>
+      </c>
+      <c r="U1136" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1136" t="s">
+        <v>2668</v>
+      </c>
+    </row>
+    <row r="1137" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1137" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1137" t="s">
+        <v>2584</v>
+      </c>
+      <c r="D1137" t="s">
+        <v>2649</v>
+      </c>
+      <c r="E1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1137" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1137" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1137" t="s">
+        <v>2650</v>
+      </c>
+      <c r="U1137" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1137" t="s">
+        <v>2669</v>
+      </c>
+    </row>
+    <row r="1138" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1138" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1138" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1138" t="s">
+        <v>2671</v>
+      </c>
+      <c r="E1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1138" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1138" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1138" t="s">
+        <v>2672</v>
+      </c>
+      <c r="U1138" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1138" t="s">
+        <v>2673</v>
+      </c>
+    </row>
+    <row r="1139" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1139" t="s">
+        <v>2566</v>
+      </c>
+      <c r="C1139" t="s">
+        <v>2584</v>
+      </c>
+      <c r="D1139" t="s">
+        <v>2674</v>
+      </c>
+      <c r="E1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1139" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1139" t="s">
+        <v>2675</v>
+      </c>
+      <c r="P1139" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1139" t="s">
+        <v>2676</v>
+      </c>
+      <c r="U1139" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1139" t="s">
+        <v>2677</v>
+      </c>
+    </row>
+    <row r="1140" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1140" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1140" t="s">
+        <v>2679</v>
+      </c>
+      <c r="D1140" t="s">
+        <v>2680</v>
+      </c>
+      <c r="E1140" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1140" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1140" t="s">
+        <v>2680</v>
+      </c>
+      <c r="H1140" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1140" t="s">
+        <v>2681</v>
+      </c>
+      <c r="P1140" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1140" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1140" t="s">
+        <v>2682</v>
+      </c>
+      <c r="T1140" t="s">
+        <v>2683</v>
+      </c>
+      <c r="U1140" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1140" t="s">
+        <v>2684</v>
+      </c>
+    </row>
+    <row r="1141" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1141" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1141" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1141" t="s">
+        <v>2686</v>
+      </c>
+      <c r="E1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1141" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1141" t="s">
+        <v>2687</v>
+      </c>
+      <c r="P1141" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1141" t="s">
+        <v>2688</v>
+      </c>
+      <c r="U1141" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1141" t="s">
+        <v>2689</v>
+      </c>
+    </row>
+    <row r="1142" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1142" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1142" t="s">
+        <v>2690</v>
+      </c>
+      <c r="D1142" t="s">
+        <v>2691</v>
+      </c>
+      <c r="E1142" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1142" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1142" t="s">
+        <v>2691</v>
+      </c>
+      <c r="H1142" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1142" t="s">
+        <v>2692</v>
+      </c>
+      <c r="P1142" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1142" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1142" t="s">
+        <v>2693</v>
+      </c>
+      <c r="T1142" t="s">
+        <v>2694</v>
+      </c>
+      <c r="U1142" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1142" t="s">
+        <v>2695</v>
+      </c>
+    </row>
+    <row r="1143" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1143" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1143" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1143" t="s">
+        <v>2300</v>
+      </c>
+      <c r="E1143" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1143" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1143" t="s">
+        <v>2300</v>
+      </c>
+      <c r="H1143" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1143" t="s">
+        <v>2696</v>
+      </c>
+      <c r="P1143" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1143" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1143" t="s">
+        <v>2697</v>
+      </c>
+      <c r="T1143" t="s">
+        <v>2698</v>
+      </c>
+      <c r="U1143" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1143" t="s">
+        <v>2699</v>
+      </c>
+    </row>
+    <row r="1144" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1144" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1144" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1144" t="s">
+        <v>2700</v>
+      </c>
+      <c r="E1144" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1144" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1144" t="s">
+        <v>2700</v>
+      </c>
+      <c r="H1144" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1144" t="s">
+        <v>2687</v>
+      </c>
+      <c r="P1144" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1144" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1144" t="s">
+        <v>2701</v>
+      </c>
+      <c r="T1144" t="s">
+        <v>2702</v>
+      </c>
+      <c r="U1144" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1144" t="s">
+        <v>2703</v>
+      </c>
+    </row>
+    <row r="1145" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1145" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1145" t="s">
+        <v>2690</v>
+      </c>
+      <c r="D1145" t="s">
+        <v>2704</v>
+      </c>
+      <c r="E1145" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1145" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1145" t="s">
+        <v>2704</v>
+      </c>
+      <c r="H1145" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1145" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1145" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1145" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1145" t="s">
+        <v>2705</v>
+      </c>
+      <c r="T1145" t="s">
+        <v>2706</v>
+      </c>
+      <c r="U1145" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1145" t="s">
+        <v>2707</v>
+      </c>
+    </row>
+    <row r="1146" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1146" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1146" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1146" t="s">
+        <v>2691</v>
+      </c>
+      <c r="E1146" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1146" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1146" t="s">
+        <v>2691</v>
+      </c>
+      <c r="H1146" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1146" t="s">
+        <v>2687</v>
+      </c>
+      <c r="P1146" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1146" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1146" t="s">
+        <v>2693</v>
+      </c>
+      <c r="T1146" t="s">
+        <v>2708</v>
+      </c>
+      <c r="U1146" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1146" t="s">
+        <v>2709</v>
+      </c>
+    </row>
+    <row r="1147" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1147" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1147" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1147" t="s">
+        <v>2710</v>
+      </c>
+      <c r="E1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1147" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1147" t="s">
+        <v>2687</v>
+      </c>
+      <c r="P1147" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1147" t="s">
+        <v>2711</v>
+      </c>
+      <c r="U1147" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1147" t="s">
+        <v>2712</v>
+      </c>
+    </row>
+    <row r="1148" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1148" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1148" t="s">
+        <v>2685</v>
+      </c>
+      <c r="D1148" t="s">
+        <v>2325</v>
+      </c>
+      <c r="E1148" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1148" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1148" t="s">
+        <v>2325</v>
+      </c>
+      <c r="H1148" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1148" t="s">
+        <v>2272</v>
+      </c>
+      <c r="P1148" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1148" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1148" t="s">
+        <v>2713</v>
+      </c>
+      <c r="T1148" t="s">
+        <v>2714</v>
+      </c>
+      <c r="U1148" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1148" t="s">
+        <v>2715</v>
+      </c>
+    </row>
+    <row r="1149" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1149" t="s">
+        <v>2678</v>
+      </c>
+      <c r="C1149" t="s">
+        <v>2716</v>
+      </c>
+      <c r="D1149" t="s">
+        <v>2717</v>
+      </c>
+      <c r="E1149" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1149" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1149" t="s">
+        <v>2717</v>
+      </c>
+      <c r="H1149" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1149" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1149" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1149" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1149" t="s">
+        <v>2705</v>
+      </c>
+      <c r="T1149" t="s">
+        <v>2706</v>
+      </c>
+      <c r="U1149" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1149" t="s">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="1150" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1150" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1150" t="s">
+        <v>2720</v>
+      </c>
+      <c r="D1150" t="s">
+        <v>2721</v>
+      </c>
+      <c r="E1150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1150" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1150" t="s">
+        <v>2721</v>
+      </c>
+      <c r="H1150" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1150" t="s">
+        <v>2722</v>
+      </c>
+      <c r="P1150" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1150" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1150" t="s">
+        <v>2723</v>
+      </c>
+      <c r="T1150" t="s">
+        <v>2724</v>
+      </c>
+      <c r="U1150" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1150" t="s">
+        <v>2725</v>
+      </c>
+    </row>
+    <row r="1151" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1151" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1151" t="s">
+        <v>2726</v>
+      </c>
+      <c r="D1151" t="s">
+        <v>2727</v>
+      </c>
+      <c r="E1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1151" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1151" t="s">
+        <v>2727</v>
+      </c>
+      <c r="H1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1151" t="s">
+        <v>2728</v>
+      </c>
+      <c r="P1151" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1151" t="s">
+        <v>2729</v>
+      </c>
+      <c r="T1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1151" t="s">
+        <v>2730</v>
+      </c>
+    </row>
+    <row r="1152" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1152" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1152" t="s">
+        <v>2731</v>
+      </c>
+      <c r="D1152" t="s">
+        <v>2732</v>
+      </c>
+      <c r="E1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1152" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1152" t="s">
+        <v>2733</v>
+      </c>
+      <c r="P1152" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1152" t="s">
+        <v>2734</v>
+      </c>
+      <c r="U1152" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1152" t="s">
+        <v>2735</v>
+      </c>
+    </row>
+    <row r="1153" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1153" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1153" t="s">
+        <v>2736</v>
+      </c>
+      <c r="D1153" t="s">
+        <v>2737</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1153" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1153" t="s">
+        <v>2738</v>
+      </c>
+      <c r="P1153" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1153" t="s">
+        <v>2739</v>
+      </c>
+      <c r="U1153" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1153" t="s">
+        <v>2740</v>
+      </c>
+    </row>
+    <row r="1154" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1154" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1154" t="s">
+        <v>2741</v>
+      </c>
+      <c r="D1154" t="s">
+        <v>2742</v>
+      </c>
+      <c r="E1154" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1154" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1154" t="s">
+        <v>2742</v>
+      </c>
+      <c r="H1154" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1154" t="s">
+        <v>2743</v>
+      </c>
+      <c r="P1154" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1154" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1154" t="s">
+        <v>2744</v>
+      </c>
+      <c r="T1154" t="s">
+        <v>2745</v>
+      </c>
+      <c r="U1154" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1154" t="s">
+        <v>2746</v>
+      </c>
+    </row>
+    <row r="1155" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1155" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1155" t="s">
+        <v>2747</v>
+      </c>
+      <c r="D1155" t="s">
+        <v>2748</v>
+      </c>
+      <c r="E1155" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1155" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1155" t="s">
+        <v>2748</v>
+      </c>
+      <c r="H1155" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1155" t="s">
+        <v>2749</v>
+      </c>
+      <c r="P1155" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1155" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1155" t="s">
+        <v>2750</v>
+      </c>
+      <c r="T1155" t="s">
+        <v>2751</v>
+      </c>
+      <c r="U1155" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1155" t="s">
+        <v>2752</v>
+      </c>
+    </row>
+    <row r="1156" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1156" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1156" t="s">
+        <v>2753</v>
+      </c>
+      <c r="D1156" t="s">
+        <v>2754</v>
+      </c>
+      <c r="E1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1156" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1156" t="s">
+        <v>2755</v>
+      </c>
+      <c r="P1156" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1156" t="s">
+        <v>2756</v>
+      </c>
+      <c r="U1156" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1156" t="s">
+        <v>2757</v>
+      </c>
+    </row>
+    <row r="1157" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1157" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1157" t="s">
+        <v>2741</v>
+      </c>
+      <c r="D1157" t="s">
+        <v>2758</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1157" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1157" t="s">
+        <v>2758</v>
+      </c>
+      <c r="H1157" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1157" t="s">
+        <v>2759</v>
+      </c>
+      <c r="P1157" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1157" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1157" t="s">
+        <v>2760</v>
+      </c>
+      <c r="T1157" t="s">
+        <v>2761</v>
+      </c>
+      <c r="U1157" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1157" t="s">
+        <v>2762</v>
+      </c>
+    </row>
+    <row r="1158" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B1158" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1158" t="s">
+        <v>2747</v>
+      </c>
+      <c r="D1158" t="s">
+        <v>2763</v>
+      </c>
+      <c r="E1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1158" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1158" t="s">
+        <v>2749</v>
+      </c>
+      <c r="P1158" t="s">
+        <v>30</v>
+      </c>
+      <c r="R1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1158" t="s">
+        <v>2764</v>
+      </c>
+      <c r="U1158" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1158" t="s">
+        <v>2765</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>